<commit_message>
update attendance and breakup marks
</commit_message>
<xml_diff>
--- a/AIAndNN/spring2026/theory/Grade/breakup.xlsx
+++ b/AIAndNN/spring2026/theory/Grade/breakup.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Air Uni\AIAndNN\spring2026\theory\Grade\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Air-Uni\AIAndNN\spring2026\theory\Grade\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F3BFB3E-7E94-432D-985E-32425F711CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A445F0BA-C5F4-49D1-A30F-18EA1199E598}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -117,7 +117,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -145,6 +145,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF5050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -176,7 +182,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -197,6 +203,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -495,18 +504,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:J9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="8.90625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.90625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.7265625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
@@ -529,24 +538,26 @@
         <v>13</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A2" s="2">
-        <v>15233</v>
+    <row r="2" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="4">
+        <v>13089</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C2" s="6">
         <v>2</v>
       </c>
       <c r="D2" s="6"/>
       <c r="E2" s="6">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-    </row>
-    <row r="3" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="G2" s="6">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="4">
         <v>14749</v>
       </c>
@@ -561,60 +572,71 @@
         <v>4.5</v>
       </c>
       <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-    </row>
-    <row r="4" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="G3" s="6">
+        <v>48</v>
+      </c>
+      <c r="J3">
+        <v>119930</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
-        <v>15147</v>
+        <v>14754</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C4" s="6">
         <v>5</v>
       </c>
       <c r="D4" s="6"/>
       <c r="E4" s="6">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-    </row>
-    <row r="5" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A5" s="4">
-        <v>13089</v>
+      <c r="G4" s="6">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="2">
+        <v>14758</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="C5" s="6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" s="6"/>
-      <c r="E5" s="6">
-        <v>4.5</v>
+      <c r="E5" s="8">
+        <v>4</v>
       </c>
       <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-    </row>
-    <row r="6" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A6" s="2">
-        <v>14754</v>
+      <c r="G5" s="6">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="5">
+        <v>14761</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" s="6">
-        <v>5</v>
+        <v>12</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>14</v>
       </c>
       <c r="D6" s="6"/>
-      <c r="E6" s="6">
+      <c r="E6" s="8">
         <v>4</v>
       </c>
       <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-    </row>
-    <row r="7" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="G6" s="6">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="4">
         <v>15025</v>
       </c>
@@ -629,39 +651,52 @@
         <v>5</v>
       </c>
       <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-    </row>
-    <row r="8" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="G7" s="6">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
-        <v>14758</v>
+        <v>15147</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="C8" s="6">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
+      <c r="E8" s="6">
+        <v>5</v>
+      </c>
       <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-    </row>
-    <row r="9" spans="1:7" ht="15.5" x14ac:dyDescent="0.35">
-      <c r="A9" s="5">
-        <v>14761</v>
+      <c r="G8" s="6">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="2">
+        <v>15233</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>14</v>
+        <v>5</v>
+      </c>
+      <c r="C9" s="6">
+        <v>2</v>
       </c>
       <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
+      <c r="E9" s="6">
+        <v>5</v>
+      </c>
       <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
+      <c r="G9" s="6">
+        <v>37</v>
+      </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G9">
+    <sortCondition ref="A1:A9"/>
+  </sortState>
   <conditionalFormatting sqref="B3">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Present">
       <formula>NOT(ISERROR(SEARCH("Present",B3)))</formula>

</xml_diff>